<commit_message>
added initial support for power cards
</commit_message>
<xml_diff>
--- a/src/main/resources/cardData.xlsx
+++ b/src/main/resources/cardData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Documents\CS491\uno3\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F873532-4B0A-4859-BBA4-BBEA8B2096DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF72327-F53B-4F33-994A-68E68D87580C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{643BDA9D-5BC1-44C5-834C-2E1825C2823B}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
   <si>
     <t>name</t>
   </si>
@@ -46,9 +46,6 @@
     <t>red 3</t>
   </si>
   <si>
-    <t xml:space="preserve"> red 40?</t>
-  </si>
-  <si>
     <t>red 4</t>
   </si>
   <si>
@@ -148,18 +145,6 @@
     <t>yellow 9</t>
   </si>
   <si>
-    <t>red Plus4</t>
-  </si>
-  <si>
-    <t>blue Plus4</t>
-  </si>
-  <si>
-    <t>green Plus4</t>
-  </si>
-  <si>
-    <t>yellow Plus4</t>
-  </si>
-  <si>
     <t>red Plus2</t>
   </si>
   <si>
@@ -199,7 +184,10 @@
     <t>spid</t>
   </si>
   <si>
-    <t>test Special</t>
+    <t>Plus 4</t>
+  </si>
+  <si>
+    <t>Wild</t>
   </si>
 </sst>
 </file>
@@ -758,169 +746,11 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="27">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="none">
           <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -940,18 +770,23 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF7C80"/>
+          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF7C80"/>
+          <bgColor rgb="FFFFCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1292,8 +1127,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7B62E53-FB95-4AD0-9DE8-D4871BF8D02A}">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -1312,7 +1150,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1356,13 +1194,10 @@
       <c r="D4" s="1">
         <v>1</v>
       </c>
-      <c r="E4" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5">
         <v>3</v>
@@ -1376,7 +1211,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6">
         <v>4</v>
@@ -1390,7 +1225,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7">
         <v>5</v>
@@ -1404,7 +1239,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8">
         <v>6</v>
@@ -1418,7 +1253,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9">
         <v>7</v>
@@ -1432,7 +1267,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10">
         <v>8</v>
@@ -1446,7 +1281,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B11">
         <v>9</v>
@@ -1460,13 +1295,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B12">
         <v>10</v>
       </c>
       <c r="C12">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D12" s="1">
         <v>1</v>
@@ -1474,13 +1309,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="B13">
         <v>11</v>
       </c>
       <c r="C13">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D13" s="1">
         <v>1</v>
@@ -1488,16 +1323,16 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="B14">
         <v>12</v>
       </c>
       <c r="C14">
-        <v>13</v>
-      </c>
-      <c r="D14" s="1">
         <v>1</v>
+      </c>
+      <c r="D14" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -1508,7 +1343,7 @@
         <v>13</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" s="2">
         <v>2</v>
@@ -1522,7 +1357,7 @@
         <v>14</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" s="2">
         <v>2</v>
@@ -1536,7 +1371,7 @@
         <v>15</v>
       </c>
       <c r="C17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D17" s="2">
         <v>2</v>
@@ -1550,7 +1385,7 @@
         <v>16</v>
       </c>
       <c r="C18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D18" s="2">
         <v>2</v>
@@ -1564,7 +1399,7 @@
         <v>17</v>
       </c>
       <c r="C19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D19" s="2">
         <v>2</v>
@@ -1578,7 +1413,7 @@
         <v>18</v>
       </c>
       <c r="C20">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D20" s="2">
         <v>2</v>
@@ -1592,7 +1427,7 @@
         <v>19</v>
       </c>
       <c r="C21">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D21" s="2">
         <v>2</v>
@@ -1606,7 +1441,7 @@
         <v>20</v>
       </c>
       <c r="C22">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D22" s="2">
         <v>2</v>
@@ -1614,13 +1449,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="B23">
         <v>21</v>
       </c>
       <c r="C23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D23" s="2">
         <v>2</v>
@@ -1628,13 +1463,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B24">
         <v>22</v>
       </c>
       <c r="C24">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D24" s="2">
         <v>2</v>
@@ -1642,13 +1477,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B25">
         <v>23</v>
       </c>
       <c r="C25">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D25" s="2">
         <v>2</v>
@@ -1656,41 +1491,41 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="B26">
         <v>24</v>
       </c>
       <c r="C26">
-        <v>12</v>
-      </c>
-      <c r="D26" s="2">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D26" s="3">
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="B27">
         <v>25</v>
       </c>
       <c r="C27">
-        <v>13</v>
-      </c>
-      <c r="D27" s="2">
         <v>2</v>
+      </c>
+      <c r="D27" s="3">
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B28">
         <v>26</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D28" s="3">
         <v>3</v>
@@ -1698,13 +1533,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B29">
         <v>27</v>
       </c>
       <c r="C29">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D29" s="3">
         <v>3</v>
@@ -1712,13 +1547,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B30">
         <v>28</v>
       </c>
       <c r="C30">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D30" s="3">
         <v>3</v>
@@ -1726,13 +1561,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B31">
         <v>29</v>
       </c>
       <c r="C31">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D31" s="3">
         <v>3</v>
@@ -1740,13 +1575,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B32">
         <v>30</v>
       </c>
       <c r="C32">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D32" s="3">
         <v>3</v>
@@ -1754,13 +1589,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B33">
         <v>31</v>
       </c>
       <c r="C33">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D33" s="3">
         <v>3</v>
@@ -1768,13 +1603,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B34">
         <v>32</v>
       </c>
       <c r="C34">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D34" s="3">
         <v>3</v>
@@ -1782,13 +1617,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="B35">
         <v>33</v>
       </c>
       <c r="C35">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D35" s="3">
         <v>3</v>
@@ -1796,13 +1631,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="B36">
         <v>34</v>
       </c>
       <c r="C36">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D36" s="3">
         <v>3</v>
@@ -1810,13 +1645,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B37">
         <v>35</v>
       </c>
       <c r="C37">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D37" s="3">
         <v>3</v>
@@ -1824,55 +1659,55 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="B38">
         <v>36</v>
       </c>
       <c r="C38">
-        <v>11</v>
-      </c>
-      <c r="D38" s="3">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="D38" s="4">
+        <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="B39">
         <v>37</v>
       </c>
       <c r="C39">
-        <v>12</v>
-      </c>
-      <c r="D39" s="3">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="D39" s="4">
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="B40">
         <v>38</v>
       </c>
       <c r="C40">
-        <v>13</v>
-      </c>
-      <c r="D40" s="3">
         <v>3</v>
+      </c>
+      <c r="D40" s="4">
+        <v>4</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B41">
         <v>39</v>
       </c>
       <c r="C41">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D41" s="4">
         <v>4</v>
@@ -1880,13 +1715,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B42">
         <v>40</v>
       </c>
       <c r="C42">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D42" s="4">
         <v>4</v>
@@ -1894,13 +1729,13 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B43">
         <v>41</v>
       </c>
       <c r="C43">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D43" s="4">
         <v>4</v>
@@ -1908,13 +1743,13 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B44">
         <v>42</v>
       </c>
       <c r="C44">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D44" s="4">
         <v>4</v>
@@ -1922,13 +1757,13 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B45">
         <v>43</v>
       </c>
       <c r="C45">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D45" s="4">
         <v>4</v>
@@ -1936,13 +1771,13 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B46">
         <v>44</v>
       </c>
       <c r="C46">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D46" s="4">
         <v>4</v>
@@ -1950,13 +1785,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B47">
         <v>45</v>
       </c>
       <c r="C47">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D47" s="4">
         <v>4</v>
@@ -1964,13 +1799,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="B48">
         <v>46</v>
       </c>
       <c r="C48">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D48" s="4">
         <v>4</v>
@@ -1978,13 +1813,13 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B49">
         <v>47</v>
       </c>
       <c r="C49">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D49" s="4">
         <v>4</v>
@@ -1992,92 +1827,106 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B50">
         <v>48</v>
       </c>
       <c r="C50">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="D50" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="B51">
         <v>49</v>
       </c>
       <c r="C51">
-        <v>11</v>
+        <v>51</v>
       </c>
       <c r="D51" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B52">
         <v>50</v>
       </c>
       <c r="C52">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="D52" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B53">
         <v>51</v>
       </c>
       <c r="C53">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="D53" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B54">
         <v>52</v>
       </c>
       <c r="C54">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D54" s="4">
-        <v>1</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>55</v>
+      </c>
+      <c r="B55">
+        <v>53</v>
+      </c>
+      <c r="C55">
+        <v>52</v>
+      </c>
+      <c r="D55" s="4">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="cellIs" dxfId="11" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
+      <formula>5</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
+      <formula>4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>3</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
+      <formula>2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="5" operator="equal">
-      <formula>2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="4" operator="equal">
-      <formula>3</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="3" operator="equal">
-      <formula>4</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
-      <formula>5</formula>
-    </cfRule>
-    <cfRule type="containsBlanks" dxfId="6" priority="7">
+    <cfRule type="containsBlanks" dxfId="0" priority="7">
       <formula>LEN(TRIM(D1))=0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
VERY basic card display testing
</commit_message>
<xml_diff>
--- a/src/main/resources/cardData.xlsx
+++ b/src/main/resources/cardData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Documents\CS491\uno3\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF72327-F53B-4F33-994A-68E68D87580C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE045E70-9987-4244-93A8-6F088C48BFA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{643BDA9D-5BC1-44C5-834C-2E1825C2823B}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="57">
   <si>
     <t>name</t>
   </si>
@@ -181,13 +181,16 @@
     <t>yellow Skip</t>
   </si>
   <si>
-    <t>spid</t>
-  </si>
-  <si>
     <t>Plus 4</t>
   </si>
   <si>
     <t>Wild</t>
+  </si>
+  <si>
+    <t>imagePath</t>
+  </si>
+  <si>
+    <t>horse.png</t>
   </si>
 </sst>
 </file>
@@ -1150,7 +1153,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1166,6 +1169,12 @@
       <c r="D2" s="1">
         <v>1</v>
       </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -1180,6 +1189,12 @@
       <c r="D3" s="1">
         <v>1</v>
       </c>
+      <c r="E3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -1194,6 +1209,12 @@
       <c r="D4" s="1">
         <v>1</v>
       </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -1208,6 +1229,12 @@
       <c r="D5" s="1">
         <v>1</v>
       </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -1222,6 +1249,12 @@
       <c r="D6" s="1">
         <v>1</v>
       </c>
+      <c r="E6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -1236,6 +1269,12 @@
       <c r="D7" s="1">
         <v>1</v>
       </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -1250,6 +1289,12 @@
       <c r="D8" s="1">
         <v>1</v>
       </c>
+      <c r="E8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -1264,6 +1309,12 @@
       <c r="D9" s="1">
         <v>1</v>
       </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -1278,6 +1329,12 @@
       <c r="D10" s="1">
         <v>1</v>
       </c>
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -1292,6 +1349,12 @@
       <c r="D11" s="1">
         <v>1</v>
       </c>
+      <c r="E11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -1306,6 +1369,12 @@
       <c r="D12" s="1">
         <v>1</v>
       </c>
+      <c r="E12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -1320,6 +1389,12 @@
       <c r="D13" s="1">
         <v>1</v>
       </c>
+      <c r="E13" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -1334,6 +1409,12 @@
       <c r="D14" s="2">
         <v>2</v>
       </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
@@ -1348,6 +1429,12 @@
       <c r="D15" s="2">
         <v>2</v>
       </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -1362,8 +1449,14 @@
       <c r="D16" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -1376,8 +1469,14 @@
       <c r="D17" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E17" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -1390,8 +1489,14 @@
       <c r="D18" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E18" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -1404,8 +1509,14 @@
       <c r="D19" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -1418,8 +1529,14 @@
       <c r="D20" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E20" t="s">
+        <v>20</v>
+      </c>
+      <c r="F20" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1432,8 +1549,14 @@
       <c r="D21" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E21" t="s">
+        <v>21</v>
+      </c>
+      <c r="F21" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1446,8 +1569,14 @@
       <c r="D22" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E22" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -1460,8 +1589,14 @@
       <c r="D23" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E23" t="s">
+        <v>42</v>
+      </c>
+      <c r="F23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>50</v>
       </c>
@@ -1474,8 +1609,14 @@
       <c r="D24" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E24" t="s">
+        <v>50</v>
+      </c>
+      <c r="F24" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>46</v>
       </c>
@@ -1488,8 +1629,14 @@
       <c r="D25" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E25" t="s">
+        <v>46</v>
+      </c>
+      <c r="F25" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -1502,8 +1649,14 @@
       <c r="D26" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>24</v>
       </c>
@@ -1516,8 +1669,14 @@
       <c r="D27" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E27" t="s">
+        <v>24</v>
+      </c>
+      <c r="F27" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>25</v>
       </c>
@@ -1530,8 +1689,14 @@
       <c r="D28" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E28" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>26</v>
       </c>
@@ -1544,8 +1709,14 @@
       <c r="D29" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E29" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>27</v>
       </c>
@@ -1558,8 +1729,14 @@
       <c r="D30" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E30" t="s">
+        <v>27</v>
+      </c>
+      <c r="F30" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>28</v>
       </c>
@@ -1572,8 +1749,14 @@
       <c r="D31" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E31" t="s">
+        <v>28</v>
+      </c>
+      <c r="F31" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>29</v>
       </c>
@@ -1586,8 +1769,14 @@
       <c r="D32" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E32" t="s">
+        <v>29</v>
+      </c>
+      <c r="F32" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>30</v>
       </c>
@@ -1600,8 +1789,14 @@
       <c r="D33" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E33" t="s">
+        <v>30</v>
+      </c>
+      <c r="F33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>31</v>
       </c>
@@ -1614,8 +1809,14 @@
       <c r="D34" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E34" t="s">
+        <v>31</v>
+      </c>
+      <c r="F34" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>43</v>
       </c>
@@ -1628,8 +1829,14 @@
       <c r="D35" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E35" t="s">
+        <v>43</v>
+      </c>
+      <c r="F35" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>51</v>
       </c>
@@ -1642,8 +1849,14 @@
       <c r="D36" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E36" t="s">
+        <v>51</v>
+      </c>
+      <c r="F36" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>47</v>
       </c>
@@ -1656,8 +1869,14 @@
       <c r="D37" s="3">
         <v>3</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E37" t="s">
+        <v>47</v>
+      </c>
+      <c r="F37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>32</v>
       </c>
@@ -1670,8 +1889,14 @@
       <c r="D38" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E38" t="s">
+        <v>32</v>
+      </c>
+      <c r="F38" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>33</v>
       </c>
@@ -1684,8 +1909,14 @@
       <c r="D39" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E39" t="s">
+        <v>33</v>
+      </c>
+      <c r="F39" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>34</v>
       </c>
@@ -1698,8 +1929,14 @@
       <c r="D40" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E40" t="s">
+        <v>34</v>
+      </c>
+      <c r="F40" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>35</v>
       </c>
@@ -1712,8 +1949,14 @@
       <c r="D41" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E41" t="s">
+        <v>35</v>
+      </c>
+      <c r="F41" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>36</v>
       </c>
@@ -1726,8 +1969,14 @@
       <c r="D42" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E42" t="s">
+        <v>36</v>
+      </c>
+      <c r="F42" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>37</v>
       </c>
@@ -1740,8 +1989,14 @@
       <c r="D43" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E43" t="s">
+        <v>37</v>
+      </c>
+      <c r="F43" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>38</v>
       </c>
@@ -1754,8 +2009,14 @@
       <c r="D44" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E44" t="s">
+        <v>38</v>
+      </c>
+      <c r="F44" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>39</v>
       </c>
@@ -1768,8 +2029,14 @@
       <c r="D45" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E45" t="s">
+        <v>39</v>
+      </c>
+      <c r="F45" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>40</v>
       </c>
@@ -1782,8 +2049,14 @@
       <c r="D46" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E46" t="s">
+        <v>40</v>
+      </c>
+      <c r="F46" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>44</v>
       </c>
@@ -1796,8 +2069,14 @@
       <c r="D47" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E47" t="s">
+        <v>44</v>
+      </c>
+      <c r="F47" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>52</v>
       </c>
@@ -1810,8 +2089,14 @@
       <c r="D48" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E48" t="s">
+        <v>52</v>
+      </c>
+      <c r="F48" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>48</v>
       </c>
@@ -1824,10 +2109,16 @@
       <c r="D49" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E49" t="s">
+        <v>48</v>
+      </c>
+      <c r="F49" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B50">
         <v>48</v>
@@ -1838,10 +2129,16 @@
       <c r="D50" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E50" t="s">
+        <v>53</v>
+      </c>
+      <c r="F50" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B51">
         <v>49</v>
@@ -1852,10 +2149,16 @@
       <c r="D51" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E51" t="s">
+        <v>53</v>
+      </c>
+      <c r="F51" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B52">
         <v>50</v>
@@ -1866,10 +2169,16 @@
       <c r="D52" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E52" t="s">
+        <v>53</v>
+      </c>
+      <c r="F52" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B53">
         <v>51</v>
@@ -1880,10 +2189,16 @@
       <c r="D53" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E53" t="s">
+        <v>53</v>
+      </c>
+      <c r="F53" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B54">
         <v>52</v>
@@ -1894,10 +2209,16 @@
       <c r="D54" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E54" t="s">
+        <v>54</v>
+      </c>
+      <c r="F54" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B55">
         <v>53</v>
@@ -1907,6 +2228,12 @@
       </c>
       <c r="D55" s="4">
         <v>5</v>
+      </c>
+      <c r="E55" t="s">
+        <v>54</v>
+      </c>
+      <c r="F55" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>